<commit_message>
fix: upload CSV for prediction gave error
</commit_message>
<xml_diff>
--- a/uploads/dataset/output/evaluasi/perbandingan_evaluasi.xlsx
+++ b/uploads/dataset/output/evaluasi/perbandingan_evaluasi.xlsx
@@ -512,10 +512,10 @@
         <v>0.06950525803508094</v>
       </c>
       <c r="K2" t="n">
-        <v>0.2655205726623535</v>
+        <v>0.4257552623748779</v>
       </c>
       <c r="L2" t="n">
-        <v>0.003075599670410156</v>
+        <v>0.004419803619384766</v>
       </c>
     </row>
     <row r="3">
@@ -552,10 +552,10 @@
         <v>0.1426562665207968</v>
       </c>
       <c r="K3" t="n">
-        <v>0.1779859066009521</v>
+        <v>0.3211314678192139</v>
       </c>
       <c r="L3" t="n">
-        <v>0.009557008743286133</v>
+        <v>0.01135730743408203</v>
       </c>
     </row>
     <row r="4">
@@ -592,10 +592,10 @@
         <v>0.1538512781550581</v>
       </c>
       <c r="K4" t="n">
-        <v>0.01423478126525879</v>
+        <v>0.002689838409423828</v>
       </c>
       <c r="L4" t="n">
-        <v>0.0005626678466796875</v>
+        <v>0.0007967948913574219</v>
       </c>
     </row>
   </sheetData>

</xml_diff>